<commit_message>
docs: refresh backlog + sprint plan xlsx
External edits from the PM track — backlog (114-story master) and
sprint plan workbook updated to reflect the Sprint 14-16 closeouts
landed on main + the in-flight DQA Rule Editor slice on the
us-076-077-079 feature branch.

Binary-only; no source impact.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/03_backlog.xlsx
+++ b/docs/03_backlog.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5899,6 +5899,277 @@
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>US-116</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>17. Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Reference Data</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>System Admin</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>As a System Admin, I want to manage choice lists (income source, education level, disability type, shock type, etc.) as versioned reference data so that I can add or retire options without touching code or Kobo.</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>- New ChoiceList and ChoiceOption models in REF-DATA with effective dates and status
+- ULID external IDs
+- Cascading lists supported via parent_code
+- Deprecate but never delete; deprecated options remain readable
+- Dual approval (author != approver) on every add/retire
+- AuditEvent on every change
+- Admin UI matching the DAT-DQA Rule Editor pattern
+- DRF endpoints under /v1/ref-data/choice-lists
+- Seed migration loads the 14 lists currently hard-coded in k-forms/build_nsr_xlsform.py</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Discussion 16 May 2026; replaces external-Kobo flow</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>Blocks US-117. Seed lists from legacy script.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>US-117</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>17. Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Intake</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>System Admin</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>As a System Admin, I want to author the questionnaire (sections, questions, skip-logic, constraints) inside the system so that the questionnaire shape, the rule pack, and the canonical schema stay in lock-step.</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>- FormSection, FormQuestion, FormSkipLogic, FormConstraint child models on FormVersion
+- FormQuestion carries type, name, label, hint, choice_list_ref, required, relevant, constraint, constraint_message, appearance, repeat_count, parameters, order_in_section
+- FormVersion immutable once activated; edits create a new version
+- Lifecycle draft → pending_approval → active → retired with dual approval
+- Custom admin UI: section/question tree on the left, edit panel on the right, drag to reorder
+- Inline validation for relevant and constraint expressions
+- One-off migration script imports the legacy questionnaire as version 1</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Discussion 16 May 2026</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>Blocks US-118, US-119, US-120 and S9 CAPI runtime.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>US-118</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>17. Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Intake</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>System Admin</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>As a System Admin, I want the system to emit a Kobo-compatible XLSForm from an active FormVersion so that the data collection tool runs the form the system designed.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>- apps/intake/xlsform/exporter.py walks a FormVersion → workbook with survey, choices, settings sheets
+- Respects every XLSForm column (type, name, label, hint, required, relevant, constraint, constraint_message, appearance, choice_filter, calculation, repeat_count, parameters)
+- select_one/select_multiple pull from referenced ChoiceList filtered by effective_from
+- Cascading geographic choice lists emitted with choice_filter
+- settings.form_id and version match FormVersion exactly
+- Output byte-for-byte deterministic
+- Round-trip test using pyxform
+- Replaces k-forms/build_nsr_xlsform.py (moved to scripts/legacy/)
+- Management command: export_xlsform --form-version &lt;id&gt;
+- REST endpoint: GET /v1/intake/form-versions/{id}/xlsform</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Discussion 16 May 2026</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Depends on US-117.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>US-119</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>17. Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Intake / DAT-DQA / DIH / DAT</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>NSR MIS</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>As the NSR MIS, I want activation of a new FormVersion to fan out to DAT-DQA, DIH MappingRules, and the canonical schema so that the rule pack, the connector mappings, and the data model never lag the questionnaire.</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>- Signal intake.form_version.activated fires inside the activation transaction
+- Listener 1 (DAT-DQA): regenerate the rule pack; rules pinned to the previous FormVersion flagged needs_review
+- Listener 2 (DIH): for every active SourceSystem, create a draft MappingRule revision pre-populated by name match; Source Admin approves before activation
+- Listener 3 (DAT): forward-only Django migration auto-generated (additive only); removed questions get deprecated_at, data preserved
+- Admin propagation screen shows fan-out status per listener
+- Activation fails atomically if any listener fails; FormVersion stays in pending_approval with the error attached
+- Tests cover add option, add question, deprecate question</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Discussion 16 May 2026</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Depends on US-117, US-118, US-076..US-079, US-106.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>US-120</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>17. Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>DIH (ING)</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Source Admin</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>As a Source Admin, I want to push a system-generated XLSForm into a Kobo project so that Kobo runs the form the system designed and there is no manual upload step.</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>- apps/ingestion_hub/connectors/kobo_push.py sibling to existing kobo.py pull connector
+- SourceSystem config: Kobo URL, project asset ID, API token (secrets manager)
+- Management command kobo_push --form-version &lt;id&gt; --source &lt;code&gt;
+- Calls Kobo asset replace endpoint and redeploys the project
+- ConnectorRun row written with mode = "push" + audit event
+- Kobo project tagged with FormVersion id; pull-side submissions link to that FormVersion automatically
+- Structured errors and Quarantine rows for invalid token, project not found, asset rejected
+- Contract tests against a stubbed Kobo server for happy path and three failure modes</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Discussion 16 May 2026</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Depends on US-118. Replaces manual XLSForm upload.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5911,7 +6182,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6333,6 +6604,30 @@
         <v>1</v>
       </c>
       <c r="F17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>17. Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Questionnaire Authoring</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" t="n">
+        <v>4</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(backlog): add US-DATA-EXP-002 — per-section synthetic samples
Backlog item for the follow-up I flagged while wiring the catalogue's
"Synthetic sample" button: have SyntheticSampleView generate a synthetic
example record for an arbitrary questionnaire SECTION (type/choice-list
aware, sensitive fields masked, deterministic per seed), not just the 8
matview-backed aggregate datasets.

- New story US-DATA-EXP-002 (Could) under a new epic "18. Data Explorer
  (DATA-EXP)"; added the matching row to the Epics sheet.
- Anonymous-accessible, flag-gated, no real household data. The catalogue
  button + ?dataset= deep-link already landed (2e8c641); this is the
  backend generator + screen support.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/03_backlog.xlsx
+++ b/docs/03_backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15320" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Epics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog'!$A$1:$I$75</definedName>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I120"/>
+  <dimension ref="A1:I121"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6170,6 +6170,57 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>US-DATA-EXP-002</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>18. Data Explorer (DATA-EXP)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Data Explorer (DATA-EXP)</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Member of the public / data requester</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>As a member of the public browsing the questionnaire catalogue, I want a synthetic (fake) example record for each questionnaire section, so I can understand the shape and meaning of the fields the registry captures before requesting access.</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>- SyntheticSampleView accepts a questionnaire section key (not only a matview-backed dataset) and returns synthetic example rows generated from the section's field metadata (type- and choice-list-aware).
+- Sensitive-class fields are masked/labelled, never populated with realistic values.
+- No real household data is read; rows are generated and deterministic per seed.
+- The catalogue 'Synthetic sample' button deep-links to the selected section's sample.
+- Anonymous-accessible (synthetic/metadata only) and behind DATA_EXPLORER_ENABLED.</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Could</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Discussion 30 May 2026 - Browse catalogue review (US-DATA-EXP-001 follow-up)</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Follow-up to US-DATA-EXP-001. Today SyntheticSampleView serves only the 8 matview-backed aggregate datasets; questionnaire sections fall back to mock. The catalogue button + ?dataset= deep-link already landed (2e8c641); this story is the backend per-section generator + screen support.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6182,7 +6233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6629,6 +6680,30 @@
       </c>
       <c r="F18" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>18. Data Explorer (DATA-EXP)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Data Explorer (DATA-EXP)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix programme detail editing and eligibility
</commit_message>
<xml_diff>
--- a/docs/03_backlog.xlsx
+++ b/docs/03_backlog.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="27040" windowHeight="15320" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Epics" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Legend" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Backlog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Epics" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Backlog'!$A$1:$I$75</definedName>
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6221,6 +6221,903 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>US-CONSENT-01</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>As a DPO, I want to create, edit and retire consent purposes with dual-approval, so the catalogue is governed.</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>- Catalogue CRUD UI under Admin &gt; Consent (SEC) &gt; Purposes
+- Dual-approval: author != approver
+- Audit events on create/activate/retire
+- API GET/POST /api/v1/consent/purposes</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>US-CONSENT-02</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>As a DPO, I want versioned, i18n statement text per purpose, so subjects always see the version they consented to.</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>- One Active version per purpose at a time
+- is_material flag forces re-consent on activation
+- Effective_from/to enforced
+- Audit events: created/activated/superseded</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>US-CONSENT-03</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Parish Chief</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>As a Parish Chief on Web, I want to capture per-purpose consent before any personal-data fields, so I comply with DPPA 2019.</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>- Pixel-match design/consent-handoff/Consent - Intake Capture.html
+- Refusal terminates intake with declined_consent outcome
+- Signature/thumbprint/verbal-witnessed/digital capture methods
+- Verbal requires witness name + role</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>US-CONSENT-04</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Field Enumerator</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>As a Field Enumerator on CAPI, I want offline consent capture with witness, so I can work without network.</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>- One question per screen
+- Offline SQLCipher store
+- Sync idempotent on (submission_id, purpose_code)
+- Witness capture works offline</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>US-CONSENT-05</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>As a citizen, I want to view my consent matrix per member, so I know how my data is used.</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>- Pixel-match Consent - Citizen Dashboard.html
+- API GET /api/v1/consent/members/{id}
+- Withdraw link only when withdrawable AND Granted
+- Locked purposes show DPPA tooltip</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>US-CONSENT-06</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Citizen</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>As a citizen, I want to request withdrawal per purpose, so I can opt out where lawful.</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>- Two-step modal: consequences then ticket confirmation
+- API POST /api/v1/consent/members/{id}/withdraw
+- Idempotent on (member, purpose, day)
+- 30-day SLA clock starts</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>US-CONSENT-07</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>As a DPO, I want a withdrawal queue with three-column detail, so I can decide each ticket within SLA.</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>- Filters: purpose, sub-region, SLA risk, channel, state
+- Decisions: Confirm, Override, Request clarification, Hold
+- Bulk Confirm: same purpose, zero referrals, max 50
+- Hourly SLA-breach alerter</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>US-CONSENT-08</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Operator</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>As an operator, I want a per-member consent badge cluster on every detail page, so I know what I can act on.</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>- 13/18 caption chips, one per purpose
+- Tooltip shows lawful basis + last change
+- Click opens AuditDrawer history
+- 60s cache acceptable</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>US-CONSENT-09</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>NSR MIS</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>As the NSR MIS, I want AC-CONSENT-* DQA rules so consent capture is enforced at validation time.</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>- AC-CONSENT-MANDATORY, METHOD-VALID, PURPOSE-VERSION-CURRENT, CAPTURE-TIMESTAMP-PLAUSIBLE, MINOR-PROXY-PRESENT seeded
+- Severities per DQA 4-tier vocab
+- DPO ratifies before activation</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>US-CONSENT-10</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Auditor</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>As an auditor, I want every consent state change in the audit chain so I can verify integrity.</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>- ConsentRecordVersion appended on every change
+- Hash chain trigger extended
+- 11 audit event types per scope §11
+- Integrity job extended to cover the new table</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>US-CONSENT-11</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>NSR MIS</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>As the NSR MIS, I want DIH promotion to write synthetic consent from the ratified DPA, so bulk imports do not bypass consent.</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>- promote_stage_record creates ConsentRecord per DPA-declared purpose
+- captured_via=DIH_FAST_TRACK, evidence=DPA PDF
+- Unratified DPA blocks promotion
+- New attestation panel in ConnectorRun detail</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>US-CONSENT-12</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>NSR MIS</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>As the NSR MIS, I want PMT recompute to respect ELIGIBILITY consent, so we do not score withdrawn members.</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>- recompute_for_household checks consent state
+- Withdrawn blocks recompute, freezes band
+- Pending re-consent blocks too
+- pmt.recompute.blocked.consent_withdrawn event emitted</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>US-CONSENT-13</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>NSR MIS</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>As the NSR MIS, I want REF candidate lists filtered at the SQL layer on REFERRAL consent, so we cannot leak by application bug.</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>- SQL clause not app-layer filter
+- Active referrals flagged for withdrawal-notify on consent loss
+- Partner programme receives structured webhook
+- Contract test green</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>US-CONSENT-14</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>As a partner, I want my DRS extract to only include rows where the purpose-mapped consent is Granted, so I do not receive non-consented data.</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>- DSA scope maps to consent purposes
+- Row-level filter on extract + preview
+- STATISTICS DSAs receive aggregates only
+- Contract test per DSA scope</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>US-CONSENT-15</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Dedup Operator</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>As a Dedup Operator, I want consent reconciled on merge, so the survivor carries the correct consent state.</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>- Union of GRANTED purposes
+- Any WITHDRAWN side -&gt; survivor WITHDRAWN
+- Conflicts surface for review and block merge
+- Reconciliation rationale in audit</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>US-CONSENT-16</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>CDO</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>As a CDO, I want head-change UPD to require new-head REGISTRATION consent, so head changes do not orphan consent.</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>- Head-change transaction routes re-capture if missing
+- Existing UPD contract tests extended
+- Audit chain preserved across head change</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>US-CONSENT-17</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>As a DPO, I want a coverage dashboard with KPIs and alerts, so I track consent health nationally.</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>- KPI cards: active REGISTRATION count, withdrawal rate, pending re-consent, average SLA, breach count
+- Alert list: SLA breaches, awaiting statement approvals, awaiting purpose approvals, DPA ratifications pending
+- Charts stubbed; KPIs live</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Should</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>US-CONSENT-18</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>NSR MIS</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>As the NSR MIS, I want the DPIA addendum and ADR-0024 published, so the build is governance-compliant.</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>- docs/dpia.md section 14 written
+- docs/adr/0024-consent-management-module.md authored
+- DPO sign-off before feature-flag flip
+- ADR references all CONSENT-O-* decisions taken</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Must</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>consent_management_scope.md §14; DPPA 2019</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Sprints S27 + S28</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I75"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6233,7 +7130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -6704,6 +7601,30 @@
       </c>
       <c r="F19" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>19. Consent Management</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Consent (SEC)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>18</v>
+      </c>
+      <c r="D20" t="n">
+        <v>17</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>